<commit_message>
Enforce physical conservation subledger ties and exclusivity
</commit_message>
<xml_diff>
--- a/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
+++ b/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6989,7 +6989,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7559,7 +7559,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8129,7 +8129,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8319,7 +8319,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8561,7 +8561,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9088,7 +9088,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9563,7 +9563,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9848,7 +9848,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10228,7 +10228,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10418,7 +10418,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10513,7 +10513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10703,7 +10703,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10798,7 +10798,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11558,7 +11558,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11653,7 +11653,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11843,7 +11843,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12128,7 +12128,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12318,7 +12318,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12413,7 +12413,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12698,7 +12698,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12888,7 +12888,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13268,7 +13268,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13363,7 +13363,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13553,7 +13553,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13838,7 +13838,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13933,7 +13933,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14218,7 +14218,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14408,7 +14408,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14693,7 +14693,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14978,7 +14978,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aaaffa9483a4f9afb971ac574aa313cd615e95ed8e404709b719da410aae14d0</t>
+          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>

<commit_message>
Complete mandated corruption detection and transaction links
</commit_message>
<xml_diff>
--- a/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
+++ b/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6989,7 +6989,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7559,7 +7559,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8129,7 +8129,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8319,7 +8319,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8561,7 +8561,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9088,7 +9088,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9563,7 +9563,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9848,7 +9848,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10228,7 +10228,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10418,7 +10418,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10513,7 +10513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10703,7 +10703,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10798,7 +10798,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11558,7 +11558,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11653,7 +11653,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11843,7 +11843,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12128,7 +12128,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12318,7 +12318,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12413,7 +12413,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12698,7 +12698,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12888,7 +12888,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13268,7 +13268,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13363,7 +13363,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13553,7 +13553,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13838,7 +13838,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13933,7 +13933,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14218,7 +14218,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14408,7 +14408,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14693,7 +14693,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14978,7 +14978,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>334b5f7ebd1a8c834f3f256cfb8f288f33516b6fbc0ecd81e83f30f5012fdf04</t>
+          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>

<commit_message>
Scale all core enterprise domains and close Part I evidence
</commit_message>
<xml_diff>
--- a/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
+++ b/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6989,7 +6989,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7559,7 +7559,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8129,7 +8129,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8319,7 +8319,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8561,7 +8561,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9088,7 +9088,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9563,7 +9563,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9848,7 +9848,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10228,7 +10228,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10418,7 +10418,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10513,7 +10513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10703,7 +10703,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10798,7 +10798,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11558,7 +11558,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11653,7 +11653,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11843,7 +11843,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12128,7 +12128,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12318,7 +12318,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12413,7 +12413,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12698,7 +12698,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12888,7 +12888,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13268,7 +13268,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13363,7 +13363,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13553,7 +13553,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13838,7 +13838,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13933,7 +13933,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14218,7 +14218,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14408,7 +14408,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14693,7 +14693,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14978,7 +14978,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f555e82108c4cbb5eaf1cc74c692abb21d28e8d8655817fa426fa5da8a7857d9</t>
+          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>

<commit_message>
Close full-scale double-entry ledger and statement lineage
</commit_message>
<xml_diff>
--- a/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
+++ b/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>-4480000</v>
+        <v>-56530000</v>
       </c>
     </row>
     <row r="38">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5789,7 +5789,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>759005000</v>
+        <v>706955000</v>
       </c>
     </row>
     <row r="38">
@@ -5804,7 +5804,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>481005000</v>
+        <v>428955000</v>
       </c>
     </row>
     <row r="39">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6345,7 +6345,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>481005000</v>
+        <v>428955000</v>
       </c>
     </row>
   </sheetData>
@@ -6419,7 +6419,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6989,7 +6989,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7559,7 +7559,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8129,7 +8129,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8319,7 +8319,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8561,7 +8561,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9088,7 +9088,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9563,7 +9563,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9848,7 +9848,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10228,7 +10228,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10418,7 +10418,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10513,7 +10513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10703,7 +10703,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10798,7 +10798,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11558,7 +11558,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11653,7 +11653,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11843,7 +11843,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12128,7 +12128,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12318,7 +12318,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12413,7 +12413,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12698,7 +12698,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12888,7 +12888,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13268,7 +13268,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13363,7 +13363,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13553,7 +13553,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13838,7 +13838,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13933,7 +13933,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14218,7 +14218,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14408,7 +14408,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14693,7 +14693,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14978,7 +14978,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628c92c722e8b67b1a3848f8d06e2bb66ae6ea4e53063d5666f5f5c0b90668bc</t>
+          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>

<commit_message>
Establish Alexandria Control public boundary v0.1.0
</commit_message>
<xml_diff>
--- a/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
+++ b/blackridge/data/public/workbooks/BLACKRIDGE_MASTER_TRACKER_v0.1.0.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6989,7 +6989,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7559,7 +7559,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8129,7 +8129,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8319,7 +8319,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>revised_correlated_downside</t>
+          <t>q4_management_valuation_case</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -8561,7 +8561,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8713,7 +8713,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>revised_correlated_downside</t>
+          <t>q4_management_valuation_case</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9088,7 +9088,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9563,7 +9563,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9848,7 +9848,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10228,7 +10228,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10418,7 +10418,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10513,7 +10513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10703,7 +10703,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10798,7 +10798,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11558,7 +11558,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11653,7 +11653,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11843,7 +11843,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12128,7 +12128,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12318,7 +12318,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12413,7 +12413,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12698,7 +12698,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12888,7 +12888,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13268,7 +13268,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13363,7 +13363,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13553,7 +13553,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13838,7 +13838,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13933,7 +13933,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14218,7 +14218,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14408,7 +14408,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14693,7 +14693,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -14978,7 +14978,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8730f8834e46889d8e7e8972e1eaa663b46f9a95dcbe01ad547ab156a7c058c9</t>
+          <t>dda9c73ec4c66e92c10410ca938c986a8a03da478ccb822044ca875bf36aa860</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>